<commit_message>
Run the second draw round for the 13 draw-recoverable strata and write the certainty-site interviews into the frame
On Jack's direct go ("run the draw for all"; "go ahead and draw" for the
certainty-site interviews). 26 Non-IDP clusters drawn and merged across
CARE, CRS, FACT, INTERSOS and Street Child (Kala/Balge drew none), and four
certainty clusters' targets raised to 05's ceiling + k: Mobbar camp 12->43,
Safana 12->17, Dan Musa 18->20, Kafur 18->19. 05: 242 -> 254 Representative.

Also fixes three defects in the post-draw projection helper that each made
a draw look better than it was (v10 paths, MSNA Light counted, MoE rounded
before comparing), and appends the new and Task 2 reinstated clusters to
partners' returned accessibility reports (36 rows).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resampling/input/accessibility_reports_returned/CARE_accessibility_report.xlsx
+++ b/resampling/input/accessibility_reports_returned/CARE_accessibility_report.xlsx
@@ -246,8 +246,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ClusterAccessibility" displayName="ClusterAccessibility" ref="A1:M256" headerRowCount="1">
-  <autoFilter ref="A1:M256"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ClusterAccessibility" displayName="ClusterAccessibility" ref="A1:M257" headerRowCount="1">
+  <autoFilter ref="A1:M257"/>
   <tableColumns count="13">
     <tableColumn id="1" name="State"/>
     <tableColumn id="2" name="LGA"/>
@@ -11758,7 +11758,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M256"/>
+  <dimension ref="A1:M257"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" style="12" min="1" max="2"/>
@@ -20373,7 +20373,6 @@
           <t>non_idp_NG026011_supp3</t>
         </is>
       </c>
-      <c r="F225" t="inlineStr"/>
       <c r="G225" t="inlineStr">
         <is>
           <t>6</t>
@@ -20411,7 +20410,6 @@
           <t>non_idp_NG008025_supp11</t>
         </is>
       </c>
-      <c r="F226" t="inlineStr"/>
       <c r="G226" t="inlineStr">
         <is>
           <t>6</t>
@@ -20449,7 +20447,6 @@
           <t>non_idp_NG021006_supp1</t>
         </is>
       </c>
-      <c r="F227" t="inlineStr"/>
       <c r="G227" t="inlineStr">
         <is>
           <t>6</t>
@@ -20487,7 +20484,6 @@
           <t>non_idp_NG008025_supp12</t>
         </is>
       </c>
-      <c r="F228" t="inlineStr"/>
       <c r="G228" t="inlineStr">
         <is>
           <t>6</t>
@@ -20525,7 +20521,6 @@
           <t>non_idp_NG008025_supp13</t>
         </is>
       </c>
-      <c r="F229" t="inlineStr"/>
       <c r="G229" t="inlineStr">
         <is>
           <t>6</t>
@@ -20563,7 +20558,6 @@
           <t>non_idp_NG008025_supp14</t>
         </is>
       </c>
-      <c r="F230" t="inlineStr"/>
       <c r="G230" t="inlineStr">
         <is>
           <t>6</t>
@@ -20601,7 +20595,6 @@
           <t>non_idp_NG008025_supp15</t>
         </is>
       </c>
-      <c r="F231" t="inlineStr"/>
       <c r="G231" t="inlineStr">
         <is>
           <t>6</t>
@@ -20639,7 +20632,6 @@
           <t>non_idp_NG008025_supp16</t>
         </is>
       </c>
-      <c r="F232" t="inlineStr"/>
       <c r="G232" t="inlineStr">
         <is>
           <t>6</t>
@@ -20677,7 +20669,6 @@
           <t>non_idp_NG026001_supp1</t>
         </is>
       </c>
-      <c r="F233" t="inlineStr"/>
       <c r="G233" t="inlineStr">
         <is>
           <t>6</t>
@@ -20715,7 +20706,6 @@
           <t>non_idp_NG026001_supp2</t>
         </is>
       </c>
-      <c r="F234" t="inlineStr"/>
       <c r="G234" t="inlineStr">
         <is>
           <t>6</t>
@@ -20753,7 +20743,6 @@
           <t>non_idp_NG026001_supp3</t>
         </is>
       </c>
-      <c r="F235" t="inlineStr"/>
       <c r="G235" t="inlineStr">
         <is>
           <t>6</t>
@@ -20791,7 +20780,6 @@
           <t>non_idp_NG026001_supp4</t>
         </is>
       </c>
-      <c r="F236" t="inlineStr"/>
       <c r="G236" t="inlineStr">
         <is>
           <t>6</t>
@@ -20829,7 +20817,6 @@
           <t>non_idp_NG026008_supp1</t>
         </is>
       </c>
-      <c r="F237" t="inlineStr"/>
       <c r="G237" t="inlineStr">
         <is>
           <t>6</t>
@@ -20867,7 +20854,6 @@
           <t>non_idp_NG022003_supp1</t>
         </is>
       </c>
-      <c r="F238" t="inlineStr"/>
       <c r="G238" t="inlineStr">
         <is>
           <t>6</t>
@@ -20905,7 +20891,6 @@
           <t>non_idp_NG022003_supp2</t>
         </is>
       </c>
-      <c r="F239" t="inlineStr"/>
       <c r="G239" t="inlineStr">
         <is>
           <t>6</t>
@@ -20943,7 +20928,6 @@
           <t>non_idp_NG022006_supp1</t>
         </is>
       </c>
-      <c r="F240" t="inlineStr"/>
       <c r="G240" t="inlineStr">
         <is>
           <t>6</t>
@@ -20981,7 +20965,6 @@
           <t>non_idp_NG022006_supp2</t>
         </is>
       </c>
-      <c r="F241" t="inlineStr"/>
       <c r="G241" t="inlineStr">
         <is>
           <t>6</t>
@@ -21019,7 +21002,6 @@
           <t>non_idp_NG022006_supp3</t>
         </is>
       </c>
-      <c r="F242" t="inlineStr"/>
       <c r="G242" t="inlineStr">
         <is>
           <t>6</t>
@@ -21057,7 +21039,6 @@
           <t>non_idp_NG022006_supp4</t>
         </is>
       </c>
-      <c r="F243" t="inlineStr"/>
       <c r="G243" t="inlineStr">
         <is>
           <t>6</t>
@@ -21095,7 +21076,6 @@
           <t>non_idp_NG008025_supp17</t>
         </is>
       </c>
-      <c r="F244" t="inlineStr"/>
       <c r="G244" t="inlineStr">
         <is>
           <t>6</t>
@@ -21611,12 +21591,50 @@
         </is>
       </c>
     </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>Borno</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Ngala</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>Ngala</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>Non-IDP</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>non_idp_NG008025_supp18</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr"/>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="I2:I256" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I257" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J256" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J257" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"N/A - fully accessible,Insecurity / conflict,Physical access (terrain, flooding, roads),Population absent / relocated,Building-footprint issue (no eligible structures),Access denied by authorities / community,Other"</formula1>
     </dataValidation>
   </dataValidations>
@@ -21625,271 +21643,4 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010064B5BF8B0F90A143B1A4ACAD04008153" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ada0274d0d067bbbdece3301958c05ce">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="30973102-2308-455b-8e1f-b6a90edc3b23" xmlns:ns3="947c1918-d5ab-48a1-8b61-0d52f2f99fd1" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f05eaaac1f596f0cf4554f8e9f637ce" ns2:_="" ns3:_="">
-    <xsd:import namespace="30973102-2308-455b-8e1f-b6a90edc3b23"/>
-    <xsd:import namespace="947c1918-d5ab-48a1-8b61-0d52f2f99fd1"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="30973102-2308-455b-8e1f-b6a90edc3b23" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="10" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="12" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="4d06f0b5-5743-41f2-90d3-b12c8ffc7f36" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="14" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="17" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="18" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="21" nillable="true" ma:displayName="Location" ma:description="" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="22" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="947c1918-d5ab-48a1-8b61-0d52f2f99fd1" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="13" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{daf5bdda-bc47-491d-9935-b3e42d5c0ae4}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="947c1918-d5ab-48a1-8b61-0d52f2f99fd1">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="19" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="20" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="30973102-2308-455b-8e1f-b6a90edc3b23">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="947c1918-d5ab-48a1-8b61-0d52f2f99fd1" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{69920729-217E-49C7-94C7-C5F7EE9B46DA}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26DDAF3C-1AC7-459E-8DDB-2A7BEE0626E9}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DFED4503-2BC6-47BB-B37C-9E53FA8124F3}"/>
 </file>
</xml_diff>